<commit_message>
scan: seg6 2026-07-24 18:52 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-24.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-24.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O125"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4343,21 +4343,21 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6641</v>
+        <v>6683</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>雍智科技</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>279.7613878118434</v>
+        <v>283.3976298280741</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>17.85</v>
+        <v>1190</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,16 +4368,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>42.8367247830634</v>
+        <v>34.26970466541711</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>13.57286708436041</v>
+        <v>22.64316373216056</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.1372495196266813</v>
+        <v>0.2362356426888746</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.0398832783644125</v>
+        <v>-42.53667416202049</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6556</v>
+        <v>6641</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>277.5429377439752</v>
+        <v>279.7613878118434</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>65.3</v>
+        <v>17.85</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>33.73026799522573</v>
+        <v>42.8367247830634</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>31.15457185899643</v>
+        <v>13.57286708436041</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.0858553499415821</v>
+        <v>0.1372495196266813</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.508162637669872</v>
+        <v>-0.0398832783644125</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6792</v>
+        <v>6556</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>詠業</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>275.6121238526458</v>
+        <v>277.5429377439752</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>53.2</v>
+        <v>65.3</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>31.85726148599029</v>
+        <v>33.73026799522573</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>22.60124358060482</v>
+        <v>31.15457185899643</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.5912007676678871</v>
+        <v>0.0858553499415821</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.6776538854339318</v>
+        <v>-0.508162637669872</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6789</v>
+        <v>6792</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>采鈺</t>
+          <t>詠業</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>274.1534449411132</v>
+        <v>275.6121238526458</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>470</v>
+        <v>53.2</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>42.92424788967899</v>
+        <v>31.85726148599029</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>12.84226388724693</v>
+        <v>22.60124358060482</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.6222333748016721</v>
+        <v>0.5912007676678871</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-3.862695751356933</v>
+        <v>-0.6776538854339318</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6624</v>
+        <v>6789</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>萬年清</t>
+          <t>采鈺</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>271.7429789063035</v>
+        <v>274.1534449411132</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>39.5</v>
+        <v>470</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>50.6092294302803</v>
+        <v>42.92424788967899</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>8.132296807141479</v>
+        <v>12.84226388724693</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.0148266642967702</v>
+        <v>0.6222333748016721</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.8531565187624032</v>
+        <v>-3.862695751356933</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6781</v>
+        <v>6624</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>萬年清</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>268.9159205525765</v>
+        <v>271.7429789063035</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>989</v>
+        <v>39.5</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>39.28760131765444</v>
+        <v>50.6092294302803</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>20.16453080876446</v>
+        <v>8.132296807141479</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.3581497768411932</v>
+        <v>0.0148266642967702</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-12.42110659936856</v>
+        <v>-0.8531565187624032</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6835</v>
+        <v>6781</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>圓裕</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>267.7113482403232</v>
+        <v>268.9159205525765</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>31.2</v>
+        <v>989</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>25.34486625843937</v>
+        <v>39.28760131765444</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>41.71224057578709</v>
+        <v>20.16453080876446</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.4084453534056392</v>
+        <v>0.3581497768411932</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.1582439039791783</v>
+        <v>-12.42110659936856</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6768</v>
+        <v>6835</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>志強-KY</t>
+          <t>圓裕</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>263.6267335297351</v>
+        <v>267.7113482403232</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>69</v>
+        <v>31.2</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>28.22531801474157</v>
+        <v>25.34486625843937</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>37.2885311865105</v>
+        <v>41.71224057578709</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>1.064935623046186</v>
+        <v>0.4084453534056392</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.2737474275934795</v>
+        <v>-0.1582439039791783</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4767,21 +4767,21 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6741</v>
+        <v>6768</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>志強-KY</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>263.3915553126218</v>
+        <v>263.6267335297351</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>32.8182539820092</v>
+        <v>28.22531801474157</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>25.2920240719063</v>
+        <v>37.2885311865105</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1.239155531262185</v>
+        <v>1.064935623046186</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.2920845310784798</v>
+        <v>0.2737474275934795</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4820,21 +4820,21 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6722</v>
+        <v>6741</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>260.6303362559336</v>
+        <v>263.3915553126218</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>34.5</v>
+        <v>55</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>43.66579018317429</v>
+        <v>32.8182539820092</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>38.4759080073088</v>
+        <v>25.2920240719063</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.521808241226955</v>
+        <v>1.239155531262185</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.1586382975020588</v>
+        <v>-0.2920845310784798</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6568</v>
+        <v>6722</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>宏觀</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>257.1956503147711</v>
+        <v>260.6303362559336</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>141</v>
+        <v>34.5</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>32.92174351422214</v>
+        <v>43.66579018317429</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>47.82032382291626</v>
+        <v>38.4759080073088</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.3927238624951129</v>
+        <v>0.521808241226955</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.4933369442522242</v>
+        <v>0.1586382975020588</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6591</v>
+        <v>6568</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>宏觀</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>256.3022092233256</v>
+        <v>257.1956503147711</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>45.3</v>
+        <v>141</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>33.88482204251814</v>
+        <v>32.92174351422214</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>41.76922837262106</v>
+        <v>47.82032382291626</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.4869869148426604</v>
+        <v>0.3927238624951129</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.29079916442398</v>
+        <v>0.4933369442522242</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6531</v>
+        <v>6591</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>255.2767283963834</v>
+        <v>256.3022092233256</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>858</v>
+        <v>45.3</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>44.52789855666523</v>
+        <v>33.88482204251814</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>15.08910880667266</v>
+        <v>41.76922837262106</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.6867829467665508</v>
+        <v>0.4869869148426604</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-3.489638716410646</v>
+        <v>-0.29079916442398</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6526</v>
+        <v>6531</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>達發</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>251.2498040747672</v>
+        <v>255.2767283963834</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>587</v>
+        <v>858</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>40.77811344881755</v>
+        <v>44.52789855666523</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>16.88655415028768</v>
+        <v>15.08910880667266</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.5198540882629474</v>
+        <v>0.6867829467665508</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-7.707988740984028</v>
+        <v>-3.489638716410646</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5085,21 +5085,21 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6725</v>
+        <v>6526</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>矽科宏晟</t>
+          <t>達發</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>247.7881440221424</v>
+        <v>251.2498040747672</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>299.5</v>
+        <v>587</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>44.2159560859647</v>
+        <v>40.77811344881755</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>13.800518705105</v>
+        <v>16.88655415028768</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.4063488233174417</v>
+        <v>0.5198540882629474</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-2.147247875626333</v>
+        <v>-7.707988740984028</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5138,21 +5138,21 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6807</v>
+        <v>6725</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>峰源-KY</t>
+          <t>矽科宏晟</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>246.0245479748466</v>
+        <v>247.7881440221424</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>33.95</v>
+        <v>299.5</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>53.85689416392397</v>
+        <v>44.2159560859647</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>12.52944419434158</v>
+        <v>13.800518705105</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.7360217208187833</v>
+        <v>0.4063488233174417</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.1166636094831229</v>
+        <v>-2.147247875626333</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6695</v>
+        <v>6807</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>峰源-KY</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>244.799554236365</v>
+        <v>246.0245479748466</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>52</v>
+        <v>33.95</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>43.95656986844109</v>
+        <v>53.85689416392397</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>14.79683474099532</v>
+        <v>12.52944419434158</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.6268839277677825</v>
+        <v>0.7360217208187833</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.4929649460099107</v>
+        <v>0.1166636094831229</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6640</v>
+        <v>6695</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>均華</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>242.1579053454525</v>
+        <v>244.799554236365</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>917</v>
+        <v>52</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,49 +5269,49 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>39.5660705927089</v>
+        <v>43.95656986844109</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>19.40673140448806</v>
+        <v>14.79683474099532</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.3844860603023584</v>
+        <v>0.6268839277677825</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M91" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>1.747908568800888</v>
+        <v>-0.4929649460099107</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6558</v>
+        <v>6640</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>239.3250664189832</v>
+        <v>242.1579053454525</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>27</v>
+        <v>917</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,49 +5322,49 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>37.23833594369891</v>
+        <v>39.5660705927089</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>23.22631948897581</v>
+        <v>19.40673140448806</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.5678981403290417</v>
+        <v>0.3844860603023584</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M92" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.1846818851252256</v>
+        <v>1.747908568800888</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6498</v>
+        <v>6727</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>久禾光</t>
+          <t>亞泰金屬</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>237.9155389555683</v>
+        <v>240.771170203729</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>79</v>
+        <v>372.5</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,16 +5375,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>30.00674994891754</v>
+        <v>42.12573877691553</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>31.35674379641715</v>
+        <v>14.97690769118036</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.5484817951580839</v>
+        <v>0.1048721020856507</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.6790237387771896</v>
+        <v>-7.718511750316605</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6698</v>
+        <v>6558</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>旭暉應材</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>237.2765678202156</v>
+        <v>239.3250664189832</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>34.7</v>
+        <v>27</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>35.92374557380734</v>
+        <v>37.23833594369891</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>20.75637866256977</v>
+        <v>23.22631948897581</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.228069749284289</v>
+        <v>0.5678981403290417</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.783523822398025</v>
+        <v>-0.1846818851252256</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6667</v>
+        <v>6498</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>233.5930660462857</v>
+        <v>237.9155389555683</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>239</v>
+        <v>79</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>35.29731734652695</v>
+        <v>30.00674994891754</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>19.21341181223953</v>
+        <v>31.35674379641715</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.5056987241134857</v>
+        <v>0.5484817951580839</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-1.823489458381572</v>
+        <v>-0.6790237387771896</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6592</v>
+        <v>6698</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>和潤企業</t>
+          <t>旭暉應材</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>230.767558744767</v>
+        <v>237.2765678202156</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>61</v>
+        <v>34.7</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>47.88095259187284</v>
+        <v>35.92374557380734</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>16.76399110154624</v>
+        <v>20.75637866256977</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.3654181420777837</v>
+        <v>0.228069749284289</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.08651479439314</v>
+        <v>-0.783523822398025</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6763</v>
+        <v>6667</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>230.7009588840838</v>
+        <v>233.5930660462857</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>42.9</v>
+        <v>239</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>39.53875278876342</v>
+        <v>35.29731734652695</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>27.93783849548544</v>
+        <v>19.21341181223953</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.379873880313373</v>
+        <v>0.5056987241134857</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.2037624956085796</v>
+        <v>-1.823489458381572</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6668</v>
+        <v>6592</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>中揚光</t>
+          <t>和潤企業</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>230.4878831409871</v>
+        <v>230.767558744767</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>33.95</v>
+        <v>61</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>33.6908768658255</v>
+        <v>47.88095259187284</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>21.26287909985419</v>
+        <v>16.76399110154624</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.5814489198712551</v>
+        <v>0.3654181420777837</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.3732944819052073</v>
+        <v>0.08651479439314</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6689</v>
+        <v>6763</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>229.6723084385925</v>
+        <v>230.7009588840838</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>60.7</v>
+        <v>42.9</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>37.63623245488745</v>
+        <v>39.53875278876342</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>21.77491089804214</v>
+        <v>27.93783849548544</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.48011294581942</v>
+        <v>0.379873880313373</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.0553793102112889</v>
+        <v>-0.2037624956085796</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5721,21 +5721,21 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6720</v>
+        <v>6668</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>久昌</t>
+          <t>中揚光</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>225.5948399055535</v>
+        <v>230.4878831409871</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>135</v>
+        <v>33.95</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>37.66870807892662</v>
+        <v>33.6908768658255</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>23.88501167831077</v>
+        <v>21.26287909985419</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.2355720869300769</v>
+        <v>0.5814489198712551</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.1487046915193683</v>
+        <v>-0.3732944819052073</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6561</v>
+        <v>6689</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>218.7155698723824</v>
+        <v>229.6723084385925</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>325.5</v>
+        <v>60.7</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>42.89057493280151</v>
+        <v>37.63623245488745</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>25.64031535075376</v>
+        <v>21.77491089804214</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.1625398832668111</v>
+        <v>0.48011294581942</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.5040395971079672</v>
+        <v>-0.0553793102112889</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5827,21 +5827,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6756</v>
+        <v>6720</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>威鋒電子</t>
+          <t>久昌</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>214.730488245691</v>
+        <v>225.5948399055535</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>97</v>
+        <v>135</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>49.51992283145621</v>
+        <v>37.66870807892662</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>19.16077987169433</v>
+        <v>23.88501167831077</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.5614204539616321</v>
+        <v>0.2355720869300769</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.3366962138139535</v>
+        <v>-0.1487046915193683</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6546</v>
+        <v>6561</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>213.6115697491381</v>
+        <v>218.7155698723824</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>59.8</v>
+        <v>325.5</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>33.50809506714592</v>
+        <v>42.89057493280151</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>28.00074000540268</v>
+        <v>25.64031535075376</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.486662816543934</v>
+        <v>0.1625398832668111</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.5697261273710588</v>
+        <v>0.5040395971079672</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5933,21 +5933,21 @@
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6690</v>
+        <v>6756</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>安碁資訊</t>
+          <t>威鋒電子</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>210.6612267653567</v>
+        <v>214.730488245691</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>162.5</v>
+        <v>97</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>42.5637267079522</v>
+        <v>49.51992283145621</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>20.48760969830276</v>
+        <v>19.16077987169433</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.4339678841670873</v>
+        <v>0.5614204539616321</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.237907209064359</v>
+        <v>-0.3366962138139535</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6512</v>
+        <v>6546</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>啟發電</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>208.8378678569989</v>
+        <v>213.6115697491381</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>20.2</v>
+        <v>59.8</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>52.55121426388861</v>
+        <v>33.50809506714592</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>9.585818301896341</v>
+        <v>28.00074000540268</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>1.12605303926152</v>
+        <v>0.486662816543934</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.901058855808857</v>
+        <v>-0.5697261273710588</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6597</v>
+        <v>6690</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>安碁資訊</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>201.7963404488422</v>
+        <v>210.6612267653567</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>60.5</v>
+        <v>162.5</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>48.29296839987801</v>
+        <v>42.5637267079522</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>9.926593865789869</v>
+        <v>20.48760969830276</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.3598643311471575</v>
+        <v>0.4339678841670873</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.1900032732574028</v>
+        <v>0.237907209064359</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6589</v>
+        <v>6512</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>台康生技</t>
+          <t>啟發電</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>199.4885029837333</v>
+        <v>208.8378678569989</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>45.6</v>
+        <v>20.2</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>46.06107983195704</v>
+        <v>52.55121426388861</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>18.05227792990141</v>
+        <v>9.585818301896341</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.2378513118894722</v>
+        <v>1.12605303926152</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.4157891398092252</v>
+        <v>0.901058855808857</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6840</v>
+        <v>6597</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>東研信超</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>197.1977710181392</v>
+        <v>201.7963404488422</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>59.9</v>
+        <v>60.5</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>39.2280862735221</v>
+        <v>48.29296839987801</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>12.58078826280035</v>
+        <v>9.926593865789869</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.3195876437674628</v>
+        <v>0.3598643311471575</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.3095308436376491</v>
+        <v>0.1900032732574028</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6605</v>
+        <v>6589</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>台康生技</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>184.8085943033747</v>
+        <v>199.4885029837333</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>132.5</v>
+        <v>45.6</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>47.55413068519616</v>
+        <v>46.06107983195704</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>14.17290039361322</v>
+        <v>18.05227792990141</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.3637893657732632</v>
+        <v>0.2378513118894722</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.3161859484809295</v>
+        <v>-0.4157891398092252</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6251,21 +6251,21 @@
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6550</v>
+        <v>6840</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>北極星藥業-KY</t>
+          <t>東研信超</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>181.8344275733412</v>
+        <v>197.1977710181392</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>12</v>
+        <v>59.9</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>36.69325289624116</v>
+        <v>39.2280862735221</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>21.13505605293864</v>
+        <v>12.58078826280035</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.69015532957411</v>
+        <v>0.3195876437674628</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0214911545496105</v>
+        <v>-0.3095308436376491</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6803</v>
+        <v>6605</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>177.8535622112384</v>
+        <v>184.8085943033747</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>274</v>
+        <v>132.5</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,16 +6329,16 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>42.96020613984566</v>
+        <v>47.55413068519616</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>46.0138309092887</v>
+        <v>14.17290039361322</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.5226278517171196</v>
+        <v>0.3637893657732632</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0161431534753901</v>
+        <v>0.3161859484809295</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6838</v>
+        <v>6550</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>北極星藥業-KY</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>176.2478737417139</v>
+        <v>181.8344275733412</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>23.8</v>
+        <v>12</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>46.07305954879097</v>
+        <v>36.69325289624116</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>9.301193326983569</v>
+        <v>21.13505605293864</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.846893190182722</v>
+        <v>0.69015532957411</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.036721310764427</v>
+        <v>-0.0214911545496105</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6708</v>
+        <v>6803</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>155.0233579256379</v>
+        <v>177.8535622112384</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>37.5</v>
+        <v>274</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>50.68033798356971</v>
+        <v>42.96020613984566</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>17.89569646195648</v>
+        <v>46.0138309092887</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.08150972309109319</v>
+        <v>0.5226278517171196</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-1.537592804918477</v>
+        <v>-0.0161431534753901</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, williams_r_recovery</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6552</v>
+        <v>6838</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>153.1963438914165</v>
+        <v>176.2478737417139</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>25.3</v>
+        <v>23.8</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>34.77835604639262</v>
+        <v>46.07305954879097</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>18.31539127977737</v>
+        <v>9.301193326983569</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.5575905863532274</v>
+        <v>0.846893190182722</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.3332855120836626</v>
+        <v>0.036721310764427</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6771</v>
+        <v>6708</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>天擎</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>152.8002475119818</v>
+        <v>155.0233579256379</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>38.5</v>
+        <v>37.5</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>38.57728175755305</v>
+        <v>50.68033798356971</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>13.23344790844882</v>
+        <v>17.89569646195648</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>2.692642779023857</v>
+        <v>0.08150972309109319</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.0341617025987679</v>
+        <v>-1.537592804918477</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, williams_r_recovery</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6794</v>
+        <v>6552</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>151.5883996077913</v>
+        <v>153.1963438914165</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>77.7</v>
+        <v>25.3</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>43.83506518263027</v>
+        <v>34.77835604639262</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>13.46440783705446</v>
+        <v>18.31539127977737</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6485196114187195</v>
+        <v>0.5575905863532274</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.2491687449162011</v>
+        <v>-0.3332855120836626</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6776</v>
+        <v>6771</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>平和環保-創</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>151.2560102937807</v>
+        <v>152.8002475119818</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>54.3</v>
+        <v>38.5</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>42.1889023811899</v>
+        <v>38.57728175755305</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>17.50901588412408</v>
+        <v>13.23344790844882</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>1.449404647562789</v>
+        <v>2.692642779023857</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.1256776387454605</v>
+        <v>0.0341617025987679</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6541</v>
+        <v>6794</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>150.1516494804123</v>
+        <v>151.5883996077913</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>38.65</v>
+        <v>77.7</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>42.75999634448463</v>
+        <v>43.83506518263027</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>11.35393296281952</v>
+        <v>13.46440783705446</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.6777723230354391</v>
+        <v>0.6485196114187195</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1431990879427314</v>
+        <v>-0.2491687449162011</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6674</v>
+        <v>6776</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>148.3296092574956</v>
+        <v>151.2560102937807</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>16</v>
+        <v>54.3</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>38.81165917491985</v>
+        <v>42.1889023811899</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.34696743352325</v>
+        <v>17.50901588412408</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.9799419874343438</v>
+        <v>1.449404647562789</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.0306288418231324</v>
+        <v>0.1256776387454605</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6796</v>
+        <v>6541</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>晉弘</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>141.2198231655696</v>
+        <v>150.1516494804123</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>58.9</v>
+        <v>38.65</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>49.31481946074547</v>
+        <v>42.75999634448463</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>14.0159975581218</v>
+        <v>11.35393296281952</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>1.059225719637045</v>
+        <v>0.6777723230354391</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.2954770980679669</v>
+        <v>-0.1431990879427314</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6823</v>
+        <v>6674</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>濾能</t>
+          <t>鋐寶科技</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>138.9674835665624</v>
+        <v>148.3296092574956</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>63.4</v>
+        <v>16</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>41.50018483648207</v>
+        <v>38.81165917491985</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>16.91373635582702</v>
+        <v>17.34696743352325</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.037723165067306</v>
+        <v>0.9799419874343438</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.2609906300596138</v>
+        <v>-0.0306288418231324</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6657</v>
+        <v>6796</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>華安</t>
+          <t>晉弘</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>109.4268861580989</v>
+        <v>141.2198231655696</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>34</v>
+        <v>58.9</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>42.3990527820528</v>
+        <v>49.31481946074547</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>18.03453384773844</v>
+        <v>14.0159975581218</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>1.391500333284305</v>
+        <v>1.059225719637045</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.0584351103776016</v>
+        <v>0.2954770980679669</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6692</v>
+        <v>6823</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>濾能</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>103.8765638555787</v>
+        <v>138.9674835665624</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>23</v>
+        <v>63.4</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>37.49175772325265</v>
+        <v>41.50018483648207</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>15.25261978889426</v>
+        <v>16.91373635582702</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.5917589028218772</v>
+        <v>1.037723165067306</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.0845953330752883</v>
+        <v>-0.2609906300596138</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -6993,21 +6993,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6625</v>
+        <v>6657</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>必應</t>
+          <t>華安</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>102.4044347631599</v>
+        <v>109.4268861580989</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>75.2</v>
+        <v>34</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>38.00497283586395</v>
+        <v>42.3990527820528</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>19.69535145014035</v>
+        <v>18.03453384773844</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.5394674845821533</v>
+        <v>1.391500333284305</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.5713185802966736</v>
+        <v>0.0584351103776016</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7046,52 +7046,158 @@
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
+        <v>6692</v>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>進能服</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>103.8765638555787</v>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H125" s="2" t="n">
+        <v>37.49175772325265</v>
+      </c>
+      <c r="I125" s="2" t="n">
+        <v>15.25261978889426</v>
+      </c>
+      <c r="J125" s="2" t="n">
+        <v>0.5917589028218772</v>
+      </c>
+      <c r="K125" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N125" s="2" t="n">
+        <v>-0.0845953330752883</v>
+      </c>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>6625</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>必應</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>102.4044347631599</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>38.00497283586395</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>19.69535145014035</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.5394674845821533</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>-0.5713185802966736</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
         <v>6614</v>
       </c>
-      <c r="B125" s="2" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
         <is>
           <t>資拓宏宇</t>
         </is>
       </c>
-      <c r="C125" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D125" s="2" t="n">
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
         <v>76.07596726553786</v>
       </c>
-      <c r="E125" s="2" t="n">
+      <c r="E127" s="2" t="n">
         <v>38.55</v>
       </c>
-      <c r="F125" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="G125" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H125" s="2" t="n">
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
         <v>39.15521521880976</v>
       </c>
-      <c r="I125" s="2" t="n">
+      <c r="I127" s="2" t="n">
         <v>16.36659101223487</v>
       </c>
-      <c r="J125" s="2" t="n">
+      <c r="J127" s="2" t="n">
         <v>0.9726780239618186</v>
       </c>
-      <c r="K125" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L125" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M125" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N125" s="2" t="n">
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
         <v>-0.1352441302225263</v>
       </c>
-      <c r="O125" s="2" t="inlineStr">
+      <c r="O127" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>